<commit_message>
Remove heroic actions and magical powers from profiles export
</commit_message>
<xml_diff>
--- a/data/raw/profiles/profiles.xlsx
+++ b/data/raw/profiles/profiles.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Profiles" sheetId="1" state="visible" r:id="rId2"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12951" uniqueCount="1738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12961" uniqueCount="1740">
   <si>
     <t xml:space="preserve">profile</t>
   </si>
@@ -5109,6 +5109,9 @@
     <t xml:space="preserve">cast</t>
   </si>
   <si>
+    <t xml:space="preserve">target</t>
+  </si>
+  <si>
     <t xml:space="preserve">instill-fear</t>
   </si>
   <si>
@@ -5172,13 +5175,16 @@
     <t xml:space="preserve">flameburst</t>
   </si>
   <si>
-    <t xml:space="preserve">fury-isengard-orc</t>
+    <t xml:space="preserve">fury</t>
+  </si>
+  <si>
+    <t xml:space="preserve">isengard-orc</t>
   </si>
   <si>
     <t xml:space="preserve">enrage-beast</t>
   </si>
   <si>
-    <t xml:space="preserve">fury-isengard-uruk-hai</t>
+    <t xml:space="preserve">isengard-uruk-hai</t>
   </si>
   <si>
     <t xml:space="preserve">bladewrath</t>
@@ -5211,7 +5217,7 @@
     <t xml:space="preserve">enchant-blades</t>
   </si>
   <si>
-    <t xml:space="preserve">fury-mordor-orc</t>
+    <t xml:space="preserve">mordor-orc</t>
   </si>
   <si>
     <t xml:space="preserve">wrath-of-bruinen</t>
@@ -5223,19 +5229,19 @@
     <t xml:space="preserve">call-winds</t>
   </si>
   <si>
-    <t xml:space="preserve">fury-beast</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fury-moria-goblin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fury-easterling</t>
+    <t xml:space="preserve">beast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">moria-goblin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">easterling</t>
   </si>
   <si>
     <t xml:space="preserve">tremor</t>
   </si>
   <si>
-    <t xml:space="preserve">fury-spider</t>
+    <t xml:space="preserve">spider</t>
   </si>
   <si>
     <t xml:space="preserve">aura-of-command</t>
@@ -5254,7 +5260,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -5276,6 +5282,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -5320,13 +5332,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -5347,13 +5363,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I571"/>
-  <sheetFormatPr defaultColWidth="8.3671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="86.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="101.5"/>
@@ -18879,7 +18895,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N571"/>
-  <sheetFormatPr defaultColWidth="8.3671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="1" width="4.64"/>
@@ -37214,7 +37230,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E739"/>
-  <sheetFormatPr defaultColWidth="8.3671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="54.9"/>
@@ -47687,11 +47703,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E200"/>
-  <sheetFormatPr defaultColWidth="8.3671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F200"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="6.65"/>
   </cols>
   <sheetData>
@@ -47711,16 +47727,19 @@
       <c r="E1" s="1" t="s">
         <v>1146</v>
       </c>
+      <c r="F1" s="0" t="s">
+        <v>1692</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>1120</v>
@@ -47734,7 +47753,7 @@
         <v>18</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1123</v>
@@ -47751,7 +47770,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>1123</v>
@@ -47768,7 +47787,7 @@
         <v>39</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>1108</v>
@@ -47785,7 +47804,7 @@
         <v>79</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>1108</v>
@@ -47802,10 +47821,10 @@
         <v>79</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>1120</v>
@@ -47819,7 +47838,7 @@
         <v>79</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>1108</v>
@@ -47836,7 +47855,7 @@
         <v>79</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>1108</v>
@@ -47853,7 +47872,7 @@
         <v>183</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>1123</v>
@@ -47870,7 +47889,7 @@
         <v>183</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>1123</v>
@@ -47887,7 +47906,7 @@
         <v>183</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>1123</v>
@@ -47904,7 +47923,7 @@
         <v>183</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>1123</v>
@@ -47921,10 +47940,10 @@
         <v>183</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>1110</v>
@@ -47938,10 +47957,10 @@
         <v>183</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>1110</v>
@@ -47955,7 +47974,7 @@
         <v>183</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>1123</v>
@@ -47972,7 +47991,7 @@
         <v>183</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>1123</v>
@@ -47989,7 +48008,7 @@
         <v>183</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>1123</v>
@@ -48006,7 +48025,7 @@
         <v>207</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>1108</v>
@@ -48023,10 +48042,10 @@
         <v>207</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>1120</v>
@@ -48040,10 +48059,10 @@
         <v>207</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>1110</v>
@@ -48057,7 +48076,7 @@
         <v>207</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>1123</v>
@@ -48074,7 +48093,7 @@
         <v>207</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>1123</v>
@@ -48091,7 +48110,7 @@
         <v>207</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>1123</v>
@@ -48108,7 +48127,7 @@
         <v>207</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>1123</v>
@@ -48125,7 +48144,7 @@
         <v>207</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>1123</v>
@@ -48142,10 +48161,10 @@
         <v>408</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>1120</v>
@@ -48159,10 +48178,10 @@
         <v>408</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>1120</v>
@@ -48176,10 +48195,10 @@
         <v>408</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>1120</v>
@@ -48193,7 +48212,7 @@
         <v>408</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>1123</v>
@@ -48210,10 +48229,10 @@
         <v>408</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>1110</v>
@@ -48227,10 +48246,10 @@
         <v>408</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>1113</v>
@@ -48244,7 +48263,7 @@
         <v>408</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>1123</v>
@@ -48261,7 +48280,7 @@
         <v>408</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>1123</v>
@@ -48278,16 +48297,19 @@
         <v>438</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E35" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>1715</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48295,7 +48317,7 @@
         <v>438</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>1714</v>
+        <v>1716</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>1108</v>
@@ -48312,7 +48334,7 @@
         <v>438</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>1123</v>
@@ -48329,7 +48351,7 @@
         <v>444</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>1123</v>
@@ -48346,10 +48368,10 @@
         <v>444</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>1120</v>
@@ -48363,7 +48385,7 @@
         <v>444</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>1123</v>
@@ -48380,16 +48402,19 @@
         <v>452</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E41" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>1717</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48397,7 +48422,7 @@
         <v>452</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>1108</v>
@@ -48414,7 +48439,7 @@
         <v>452</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>1123</v>
@@ -48431,7 +48456,7 @@
         <v>515</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>1108</v>
@@ -48448,10 +48473,10 @@
         <v>515</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>1120</v>
@@ -48465,10 +48490,10 @@
         <v>515</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>1110</v>
@@ -48482,7 +48507,7 @@
         <v>515</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>1123</v>
@@ -48499,7 +48524,7 @@
         <v>515</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>1123</v>
@@ -48516,7 +48541,7 @@
         <v>515</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>1123</v>
@@ -48533,7 +48558,7 @@
         <v>515</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>1123</v>
@@ -48550,7 +48575,7 @@
         <v>515</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>1123</v>
@@ -48567,7 +48592,7 @@
         <v>548</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>1717</v>
+        <v>1719</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>1123</v>
@@ -48584,7 +48609,7 @@
         <v>548</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>1718</v>
+        <v>1720</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>1123</v>
@@ -48601,10 +48626,10 @@
         <v>548</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>1110</v>
@@ -48618,7 +48643,7 @@
         <v>552</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>1719</v>
+        <v>1721</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>1123</v>
@@ -48635,10 +48660,10 @@
         <v>552</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>1120</v>
@@ -48652,7 +48677,7 @@
         <v>552</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>1123</v>
@@ -48669,7 +48694,7 @@
         <v>552</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>1720</v>
+        <v>1722</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>1123</v>
@@ -48686,10 +48711,10 @@
         <v>552</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>1721</v>
+        <v>1723</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>1113</v>
@@ -48703,10 +48728,10 @@
         <v>552</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>1113</v>
@@ -48720,10 +48745,10 @@
         <v>552</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>1723</v>
+        <v>1725</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>1113</v>
@@ -48737,10 +48762,10 @@
         <v>556</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>1120</v>
@@ -48754,10 +48779,10 @@
         <v>556</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>1120</v>
@@ -48771,7 +48796,7 @@
         <v>556</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>1123</v>
@@ -48788,10 +48813,10 @@
         <v>556</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>1120</v>
@@ -48805,10 +48830,10 @@
         <v>556</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D66" s="1" t="s">
         <v>1120</v>
@@ -48822,10 +48847,10 @@
         <v>556</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D67" s="1" t="s">
         <v>1110</v>
@@ -48839,7 +48864,7 @@
         <v>556</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>1123</v>
@@ -48856,7 +48881,7 @@
         <v>634</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>1123</v>
@@ -48873,7 +48898,7 @@
         <v>634</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>1123</v>
@@ -48890,7 +48915,7 @@
         <v>634</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>1123</v>
@@ -48907,7 +48932,7 @@
         <v>638</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>1123</v>
@@ -48924,7 +48949,7 @@
         <v>638</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>1123</v>
@@ -48941,7 +48966,7 @@
         <v>638</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>1123</v>
@@ -48958,7 +48983,7 @@
         <v>638</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>1108</v>
@@ -48975,10 +49000,10 @@
         <v>638</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>1114</v>
@@ -48992,10 +49017,10 @@
         <v>647</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>1120</v>
@@ -49009,10 +49034,10 @@
         <v>647</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D78" s="1" t="s">
         <v>1120</v>
@@ -49026,10 +49051,10 @@
         <v>647</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>1120</v>
@@ -49043,7 +49068,7 @@
         <v>647</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>1123</v>
@@ -49060,10 +49085,10 @@
         <v>647</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>1110</v>
@@ -49077,10 +49102,10 @@
         <v>647</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>1113</v>
@@ -49094,7 +49119,7 @@
         <v>651</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>1123</v>
@@ -49111,7 +49136,7 @@
         <v>651</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>1123</v>
@@ -49128,7 +49153,7 @@
         <v>651</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>1123</v>
@@ -49145,7 +49170,7 @@
         <v>651</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>1123</v>
@@ -49162,7 +49187,7 @@
         <v>651</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>1108</v>
@@ -49179,10 +49204,10 @@
         <v>651</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>1113</v>
@@ -49196,7 +49221,7 @@
         <v>651</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>1123</v>
@@ -49213,16 +49238,19 @@
         <v>659</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>1726</v>
+        <v>1714</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E90" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>1728</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -49230,7 +49258,7 @@
         <v>659</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>1123</v>
@@ -49247,7 +49275,7 @@
         <v>659</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>1123</v>
@@ -49264,10 +49292,10 @@
         <v>686</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>1120</v>
@@ -49281,10 +49309,10 @@
         <v>686</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>1120</v>
@@ -49298,7 +49326,7 @@
         <v>686</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>1123</v>
@@ -49315,7 +49343,7 @@
         <v>686</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>1123</v>
@@ -49332,7 +49360,7 @@
         <v>686</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>1717</v>
+        <v>1719</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>1123</v>
@@ -49349,7 +49377,7 @@
         <v>686</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>1123</v>
@@ -49366,7 +49394,7 @@
         <v>686</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>1718</v>
+        <v>1720</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>1123</v>
@@ -49383,7 +49411,7 @@
         <v>686</v>
       </c>
       <c r="B100" s="0" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>1123</v>
@@ -49400,7 +49428,7 @@
         <v>686</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>1123</v>
@@ -49417,7 +49445,7 @@
         <v>734</v>
       </c>
       <c r="B102" s="0" t="s">
-        <v>1720</v>
+        <v>1722</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>1123</v>
@@ -49434,10 +49462,10 @@
         <v>734</v>
       </c>
       <c r="B103" s="0" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="D103" s="1" t="s">
         <v>1110</v>
@@ -49451,7 +49479,7 @@
         <v>739</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>1123</v>
@@ -49468,10 +49496,10 @@
         <v>739</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>1110</v>
@@ -49485,7 +49513,7 @@
         <v>739</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>1108</v>
@@ -49502,10 +49530,10 @@
         <v>739</v>
       </c>
       <c r="B107" s="0" t="s">
-        <v>1723</v>
+        <v>1725</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D107" s="1" t="s">
         <v>1110</v>
@@ -49519,10 +49547,10 @@
         <v>741</v>
       </c>
       <c r="B108" s="0" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D108" s="1" t="s">
         <v>1120</v>
@@ -49536,7 +49564,7 @@
         <v>741</v>
       </c>
       <c r="B109" s="0" t="s">
-        <v>1728</v>
+        <v>1730</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>1108</v>
@@ -49553,7 +49581,7 @@
         <v>741</v>
       </c>
       <c r="B110" s="0" t="s">
-        <v>1729</v>
+        <v>1731</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>1123</v>
@@ -49570,7 +49598,7 @@
         <v>741</v>
       </c>
       <c r="B111" s="0" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>1108</v>
@@ -49587,10 +49615,10 @@
         <v>741</v>
       </c>
       <c r="B112" s="0" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D112" s="1" t="s">
         <v>1113</v>
@@ -49604,7 +49632,7 @@
         <v>744</v>
       </c>
       <c r="B113" s="0" t="s">
-        <v>1720</v>
+        <v>1722</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>1123</v>
@@ -49621,10 +49649,10 @@
         <v>744</v>
       </c>
       <c r="B114" s="0" t="s">
-        <v>1727</v>
+        <v>1729</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="D114" s="1" t="s">
         <v>1110</v>
@@ -49638,7 +49666,7 @@
         <v>750</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>1123</v>
@@ -49655,7 +49683,7 @@
         <v>750</v>
       </c>
       <c r="B116" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>1123</v>
@@ -49672,7 +49700,7 @@
         <v>750</v>
       </c>
       <c r="B117" s="0" t="s">
-        <v>1728</v>
+        <v>1730</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>1123</v>
@@ -49689,10 +49717,10 @@
         <v>750</v>
       </c>
       <c r="B118" s="0" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D118" s="1" t="s">
         <v>1110</v>
@@ -49706,10 +49734,10 @@
         <v>750</v>
       </c>
       <c r="B119" s="0" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D119" s="1" t="s">
         <v>1110</v>
@@ -49723,7 +49751,7 @@
         <v>750</v>
       </c>
       <c r="B120" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>1123</v>
@@ -49740,7 +49768,7 @@
         <v>759</v>
       </c>
       <c r="B121" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>1108</v>
@@ -49757,7 +49785,7 @@
         <v>759</v>
       </c>
       <c r="B122" s="0" t="s">
-        <v>1720</v>
+        <v>1722</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>1108</v>
@@ -49774,7 +49802,7 @@
         <v>852</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>1123</v>
@@ -49791,7 +49819,7 @@
         <v>852</v>
       </c>
       <c r="B124" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>1123</v>
@@ -49808,7 +49836,7 @@
         <v>852</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>1123</v>
@@ -49825,7 +49853,7 @@
         <v>855</v>
       </c>
       <c r="B126" s="0" t="s">
-        <v>1714</v>
+        <v>1716</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>1108</v>
@@ -49842,16 +49870,19 @@
         <v>855</v>
       </c>
       <c r="B127" s="0" t="s">
-        <v>1730</v>
+        <v>1714</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D127" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E127" s="1" t="n">
         <v>2</v>
+      </c>
+      <c r="F127" s="0" t="s">
+        <v>1732</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -49859,10 +49890,10 @@
         <v>855</v>
       </c>
       <c r="B128" s="0" t="s">
-        <v>1723</v>
+        <v>1725</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D128" s="1" t="s">
         <v>1110</v>
@@ -49876,16 +49907,19 @@
         <v>862</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>1731</v>
+        <v>1714</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D129" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E129" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>1733</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -49893,10 +49927,10 @@
         <v>862</v>
       </c>
       <c r="B130" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D130" s="1" t="s">
         <v>1110</v>
@@ -49910,7 +49944,7 @@
         <v>862</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>1123</v>
@@ -49927,7 +49961,7 @@
         <v>892</v>
       </c>
       <c r="B132" s="0" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>1123</v>
@@ -49944,16 +49978,19 @@
         <v>892</v>
       </c>
       <c r="B133" s="0" t="s">
-        <v>1732</v>
+        <v>1714</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E133" s="1" t="n">
         <v>2</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>1734</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -49961,7 +49998,7 @@
         <v>892</v>
       </c>
       <c r="B134" s="0" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>1123</v>
@@ -49978,10 +50015,10 @@
         <v>892</v>
       </c>
       <c r="B135" s="0" t="s">
-        <v>1733</v>
+        <v>1735</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D135" s="1" t="s">
         <v>1113</v>
@@ -49995,7 +50032,7 @@
         <v>900</v>
       </c>
       <c r="B136" s="0" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>1108</v>
@@ -50012,16 +50049,19 @@
         <v>900</v>
       </c>
       <c r="B137" s="0" t="s">
-        <v>1732</v>
+        <v>1714</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D137" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E137" s="1" t="n">
         <v>2</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>1734</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -50029,7 +50069,7 @@
         <v>900</v>
       </c>
       <c r="B138" s="0" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>1108</v>
@@ -50046,7 +50086,7 @@
         <v>933</v>
       </c>
       <c r="B139" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>1123</v>
@@ -50063,7 +50103,7 @@
         <v>933</v>
       </c>
       <c r="B140" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>1123</v>
@@ -50080,7 +50120,7 @@
         <v>933</v>
       </c>
       <c r="B141" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>1123</v>
@@ -50097,7 +50137,7 @@
         <v>970</v>
       </c>
       <c r="B142" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>1123</v>
@@ -50114,10 +50154,10 @@
         <v>970</v>
       </c>
       <c r="B143" s="0" t="s">
-        <v>1723</v>
+        <v>1725</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D143" s="1" t="s">
         <v>1110</v>
@@ -50131,7 +50171,7 @@
         <v>982</v>
       </c>
       <c r="B144" s="0" t="s">
-        <v>1729</v>
+        <v>1731</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>1123</v>
@@ -50148,7 +50188,7 @@
         <v>982</v>
       </c>
       <c r="B145" s="0" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>1123</v>
@@ -50165,10 +50205,10 @@
         <v>982</v>
       </c>
       <c r="B146" s="0" t="s">
-        <v>1723</v>
+        <v>1725</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D146" s="1" t="s">
         <v>1110</v>
@@ -50182,7 +50222,7 @@
         <v>988</v>
       </c>
       <c r="B147" s="0" t="s">
-        <v>1729</v>
+        <v>1731</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>1123</v>
@@ -50199,7 +50239,7 @@
         <v>988</v>
       </c>
       <c r="B148" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>1123</v>
@@ -50216,7 +50256,7 @@
         <v>988</v>
       </c>
       <c r="B149" s="0" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>1123</v>
@@ -50233,16 +50273,19 @@
         <v>994</v>
       </c>
       <c r="B150" s="0" t="s">
-        <v>1734</v>
+        <v>1714</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D150" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E150" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>1736</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -50250,7 +50293,7 @@
         <v>994</v>
       </c>
       <c r="B151" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>1123</v>
@@ -50267,7 +50310,7 @@
         <v>1033</v>
       </c>
       <c r="B152" s="0" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>1108</v>
@@ -50284,16 +50327,19 @@
         <v>1033</v>
       </c>
       <c r="B153" s="0" t="s">
-        <v>1726</v>
+        <v>1714</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D153" s="1" t="s">
         <v>1120</v>
       </c>
       <c r="E153" s="1" t="n">
         <v>2</v>
+      </c>
+      <c r="F153" s="0" t="s">
+        <v>1728</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -50301,7 +50347,7 @@
         <v>1034</v>
       </c>
       <c r="B154" s="0" t="s">
-        <v>1716</v>
+        <v>1718</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>1123</v>
@@ -50318,7 +50364,7 @@
         <v>1034</v>
       </c>
       <c r="B155" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>1123</v>
@@ -50335,7 +50381,7 @@
         <v>1034</v>
       </c>
       <c r="B156" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>1123</v>
@@ -50352,7 +50398,7 @@
         <v>1034</v>
       </c>
       <c r="B157" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>1123</v>
@@ -50369,7 +50415,7 @@
         <v>1034</v>
       </c>
       <c r="B158" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>1108</v>
@@ -50386,10 +50432,10 @@
         <v>1034</v>
       </c>
       <c r="B159" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D159" s="1" t="s">
         <v>1114</v>
@@ -50403,7 +50449,7 @@
         <v>1058</v>
       </c>
       <c r="B160" s="0" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>1108</v>
@@ -50420,10 +50466,10 @@
         <v>1058</v>
       </c>
       <c r="B161" s="0" t="s">
-        <v>1733</v>
+        <v>1735</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D161" s="1" t="s">
         <v>1113</v>
@@ -50437,7 +50483,7 @@
         <v>1060</v>
       </c>
       <c r="B162" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>1123</v>
@@ -50454,7 +50500,7 @@
         <v>1060</v>
       </c>
       <c r="B163" s="0" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>1123</v>
@@ -50471,7 +50517,7 @@
         <v>1060</v>
       </c>
       <c r="B164" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>1123</v>
@@ -50488,7 +50534,7 @@
         <v>1067</v>
       </c>
       <c r="B165" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>1123</v>
@@ -50505,7 +50551,7 @@
         <v>1067</v>
       </c>
       <c r="B166" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>1123</v>
@@ -50522,7 +50568,7 @@
         <v>1067</v>
       </c>
       <c r="B167" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>1123</v>
@@ -50539,7 +50585,7 @@
         <v>1067</v>
       </c>
       <c r="B168" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>1108</v>
@@ -50556,7 +50602,7 @@
         <v>1067</v>
       </c>
       <c r="B169" s="0" t="s">
-        <v>1719</v>
+        <v>1721</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>1123</v>
@@ -50573,10 +50619,10 @@
         <v>1067</v>
       </c>
       <c r="B170" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D170" s="1" t="s">
         <v>1114</v>
@@ -50590,10 +50636,10 @@
         <v>1069</v>
       </c>
       <c r="B171" s="0" t="s">
-        <v>1735</v>
+        <v>1737</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D171" s="1" t="s">
         <v>1120</v>
@@ -50607,7 +50653,7 @@
         <v>1069</v>
       </c>
       <c r="B172" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>1123</v>
@@ -50624,7 +50670,7 @@
         <v>1069</v>
       </c>
       <c r="B173" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>1123</v>
@@ -50641,7 +50687,7 @@
         <v>1069</v>
       </c>
       <c r="B174" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>1123</v>
@@ -50658,7 +50704,7 @@
         <v>1069</v>
       </c>
       <c r="B175" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>1108</v>
@@ -50675,10 +50721,10 @@
         <v>1069</v>
       </c>
       <c r="B176" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D176" s="1" t="s">
         <v>1114</v>
@@ -50692,7 +50738,7 @@
         <v>1070</v>
       </c>
       <c r="B177" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C177" s="1" t="s">
         <v>1123</v>
@@ -50709,7 +50755,7 @@
         <v>1070</v>
       </c>
       <c r="B178" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>1123</v>
@@ -50726,7 +50772,7 @@
         <v>1070</v>
       </c>
       <c r="B179" s="0" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>1123</v>
@@ -50743,7 +50789,7 @@
         <v>1070</v>
       </c>
       <c r="B180" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C180" s="1" t="s">
         <v>1123</v>
@@ -50760,7 +50806,7 @@
         <v>1070</v>
       </c>
       <c r="B181" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>1108</v>
@@ -50777,10 +50823,10 @@
         <v>1070</v>
       </c>
       <c r="B182" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D182" s="1" t="s">
         <v>1114</v>
@@ -50794,7 +50840,7 @@
         <v>1073</v>
       </c>
       <c r="B183" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>1123</v>
@@ -50811,7 +50857,7 @@
         <v>1073</v>
       </c>
       <c r="B184" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C184" s="1" t="s">
         <v>1123</v>
@@ -50828,7 +50874,7 @@
         <v>1073</v>
       </c>
       <c r="B185" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C185" s="1" t="s">
         <v>1123</v>
@@ -50845,7 +50891,7 @@
         <v>1073</v>
       </c>
       <c r="B186" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C186" s="1" t="s">
         <v>1108</v>
@@ -50862,7 +50908,7 @@
         <v>1073</v>
       </c>
       <c r="B187" s="0" t="s">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>1123</v>
@@ -50879,10 +50925,10 @@
         <v>1073</v>
       </c>
       <c r="B188" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C188" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D188" s="1" t="s">
         <v>1114</v>
@@ -50896,7 +50942,7 @@
         <v>1074</v>
       </c>
       <c r="B189" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>1123</v>
@@ -50913,10 +50959,10 @@
         <v>1074</v>
       </c>
       <c r="B190" s="0" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D190" s="1" t="s">
         <v>1120</v>
@@ -50930,7 +50976,7 @@
         <v>1074</v>
       </c>
       <c r="B191" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C191" s="1" t="s">
         <v>1123</v>
@@ -50947,7 +50993,7 @@
         <v>1074</v>
       </c>
       <c r="B192" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C192" s="1" t="s">
         <v>1123</v>
@@ -50964,7 +51010,7 @@
         <v>1074</v>
       </c>
       <c r="B193" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C193" s="1" t="s">
         <v>1108</v>
@@ -50981,10 +51027,10 @@
         <v>1074</v>
       </c>
       <c r="B194" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C194" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D194" s="1" t="s">
         <v>1114</v>
@@ -50998,7 +51044,7 @@
         <v>1081</v>
       </c>
       <c r="B195" s="0" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C195" s="1" t="s">
         <v>1123</v>
@@ -51015,7 +51061,7 @@
         <v>1081</v>
       </c>
       <c r="B196" s="0" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="C196" s="1" t="s">
         <v>1123</v>
@@ -51032,7 +51078,7 @@
         <v>1081</v>
       </c>
       <c r="B197" s="0" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="C197" s="1" t="s">
         <v>1123</v>
@@ -51049,7 +51095,7 @@
         <v>1081</v>
       </c>
       <c r="B198" s="0" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="C198" s="1" t="s">
         <v>1123</v>
@@ -51066,7 +51112,7 @@
         <v>1081</v>
       </c>
       <c r="B199" s="0" t="s">
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="C199" s="1" t="s">
         <v>1108</v>
@@ -51083,10 +51129,10 @@
         <v>1081</v>
       </c>
       <c r="B200" s="0" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="D200" s="1" t="s">
         <v>1114</v>
@@ -51112,7 +51158,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.3671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35.23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.66"/>
@@ -51124,7 +51170,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1736</v>
+        <v>1738</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1146</v>
@@ -51135,7 +51181,7 @@
         <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>1</v>
@@ -51146,7 +51192,7 @@
         <v>128</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>1</v>
@@ -51157,7 +51203,7 @@
         <v>198</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>1</v>
@@ -51168,7 +51214,7 @@
         <v>261</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>1</v>
@@ -51179,7 +51225,7 @@
         <v>295</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>1</v>
@@ -51190,7 +51236,7 @@
         <v>299</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>1</v>
@@ -51201,7 +51247,7 @@
         <v>314</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>1</v>
@@ -51212,7 +51258,7 @@
         <v>321</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>1</v>
@@ -51223,7 +51269,7 @@
         <v>431</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>1</v>
@@ -51234,7 +51280,7 @@
         <v>434</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>1</v>
@@ -51245,7 +51291,7 @@
         <v>457</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>1</v>
@@ -51256,7 +51302,7 @@
         <v>486</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -51267,7 +51313,7 @@
         <v>488</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>1</v>
@@ -51278,7 +51324,7 @@
         <v>585</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>1</v>
@@ -51289,7 +51335,7 @@
         <v>588</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>1</v>
@@ -51300,7 +51346,7 @@
         <v>603</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C17" s="1" t="n">
         <v>1</v>
@@ -51311,7 +51357,7 @@
         <v>629</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
@@ -51322,7 +51368,7 @@
         <v>656</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
@@ -51333,7 +51379,7 @@
         <v>687</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>1</v>
@@ -51344,7 +51390,7 @@
         <v>725</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C21" s="1" t="n">
         <v>1</v>
@@ -51355,7 +51401,7 @@
         <v>739</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>1</v>
@@ -51366,7 +51412,7 @@
         <v>750</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C23" s="1" t="n">
         <v>1</v>
@@ -51377,7 +51423,7 @@
         <v>752</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C24" s="1" t="n">
         <v>1</v>
@@ -51388,7 +51434,7 @@
         <v>830</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C25" s="1" t="n">
         <v>1</v>
@@ -51399,7 +51445,7 @@
         <v>864</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C26" s="1" t="n">
         <v>1</v>
@@ -51410,7 +51456,7 @@
         <v>1088</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>1737</v>
+        <v>1739</v>
       </c>
       <c r="C27" s="1" t="n">
         <v>1</v>

</xml_diff>